<commit_message>
CMS Overhaul: SQLite, dynamic page-wise edit tabs, navigation ordering, and support/contact detail editors
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -399,10 +399,87 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetData/>
+  <dimension ref="A1:J2"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="8" max="8" width="40.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>First Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Last Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Organization</v>
+      </c>
+      <c r="D1" t="str">
+        <v>City</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Email ID</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Mobile No.</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Subject</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Message</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Terms Accepted</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Submitted At</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Test</v>
+      </c>
+      <c r="B2" t="str">
+        <v>User</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Test Org</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Test City</v>
+      </c>
+      <c r="E2" t="str">
+        <v>test.user@rockmix.com</v>
+      </c>
+      <c r="F2" t="str">
+        <v>9999988888</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Test Subject</v>
+      </c>
+      <c r="H2" t="str">
+        <v>This is a test message to verify SQLite lead tracking.</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-07-06T08:54:07.752Z</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>